<commit_message>
feat: categorie-detectie per artikel (Voedsel/Drank/Alcohol/...) + Groq vision + Excel met categorie-kolommen
</commit_message>
<xml_diff>
--- a/bonnen.xlsx
+++ b/bonnen.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
   <si>
     <t>Datum</t>
   </si>
@@ -21,64 +21,70 @@
     <t>Week</t>
   </si>
   <si>
-    <t>Thema</t>
-  </si>
-  <si>
     <t>Winkel</t>
   </si>
   <si>
-    <t>Bedrag</t>
-  </si>
-  <si>
-    <t>Omschrijving</t>
-  </si>
-  <si>
-    <t>Ingescand</t>
+    <t>Voedsel</t>
+  </si>
+  <si>
+    <t>Drank</t>
+  </si>
+  <si>
+    <t>Alcohol</t>
+  </si>
+  <si>
+    <t>Spelmateriaal</t>
+  </si>
+  <si>
+    <t>Knutselgerief</t>
+  </si>
+  <si>
+    <t>Kuisproducten</t>
+  </si>
+  <si>
+    <t>Varia</t>
+  </si>
+  <si>
+    <t>Totaal</t>
   </si>
   <si>
     <t>Fingerprint</t>
   </si>
   <si>
-    <t>Overzicht per week en thema</t>
+    <t>Overzicht per week en categorie</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>Jungle</t>
-  </si>
-  <si>
-    <t>Ruimte</t>
-  </si>
-  <si>
-    <t>Piraten</t>
-  </si>
-  <si>
-    <t>Middeleeuwen</t>
-  </si>
-  <si>
-    <t>Superhelden</t>
-  </si>
-  <si>
     <t>TOTAAL</t>
   </si>
   <si>
-    <t>Week 1 (7–11 jul)</t>
-  </si>
-  <si>
-    <t>Week 2 (14–18 jul)</t>
-  </si>
-  <si>
-    <t>Week 3 (21–25 jul)</t>
-  </si>
-  <si>
-    <t>Week 4 (28 jul–1 aug)</t>
-  </si>
-  <si>
-    <t>Week 5 (4–8 aug)</t>
-  </si>
-  <si>
-    <t>Week 6 (11–15 aug)</t>
+    <t>Opbouw</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Week 7</t>
+  </si>
+  <si>
+    <t>Afbraak</t>
   </si>
   <si>
     <t>Speelplein-kassa — handleiding</t>
@@ -87,40 +93,46 @@
     <t>HOE WERKT HET?</t>
   </si>
   <si>
-    <t>1. Open de scan-app op je telefoon (link ontvangen van de organisatie).</t>
+    <t>1. Open de scan-app op je telefoon (link van de organisatie).</t>
   </si>
   <si>
     <t>2. Tik "Scan een bonnetje" en neem een foto van de kassabon.</t>
   </si>
   <si>
-    <t>3. Controleer de ingevulde gegevens (datum, bedrag, winkel).</t>
-  </si>
-  <si>
-    <t>4. Kies het juiste thema en de week.</t>
-  </si>
-  <si>
-    <t>5. Tik "Bewaar in Excel" — de bon komt automatisch hier in het tabblad Data.</t>
+    <t>3. De AI leest elk artikel uit en kiest automatisch een categorie.</t>
+  </si>
+  <si>
+    <t>4. Controleer de categorieën (tik erop om te wijzigen) en het totaal.</t>
+  </si>
+  <si>
+    <t>5. Tik "Bewaar in Excel" — de bon komt automatisch in het tabblad Data.</t>
+  </si>
+  <si>
+    <t>CATEGORIEËN</t>
+  </si>
+  <si>
+    <t>Voedsel, Drank, Alcohol, Spelmateriaal, Knutselgerief, Kuisproducten, Varia.</t>
+  </si>
+  <si>
+    <t>Het totaalbedrag wordt over deze categorie-kolommen verdeeld.</t>
   </si>
   <si>
     <t>DUBBELE BONNEN</t>
   </si>
   <si>
-    <t>Als je dezelfde bon twee keer scant, krijg je een foutmelding. De bon wordt niet dubbel opgeslagen.</t>
+    <t>Dezelfde bon (winkel + datum + bedrag) twee keer scannen wordt geweigerd.</t>
   </si>
   <si>
     <t>OVERZICHT</t>
   </si>
   <si>
-    <t>Tabblad Overzicht toont de totalen per week en per thema. Die berekent Excel automatisch.</t>
+    <t>Tabblad Overzicht telt automatisch per week en per categorie op.</t>
   </si>
   <si>
     <t>LET OP</t>
   </si>
   <si>
-    <t>Verander de naam van de tabel (Bonnen) of de kolomtitels NIET.</t>
-  </si>
-  <si>
-    <t>De app verwacht exact die namen.</t>
+    <t>Verander de tabelnaam (Bonnen) of de kolomtitels NIET.</t>
   </si>
 </sst>
 </file>
@@ -140,12 +152,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF2F8F5B"/>
+      <sz val="14"/>
     </font>
     <font>
       <b/>
-      <color rgb="FF4F6EF7"/>
-      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
     </font>
     <font>
       <b/>
@@ -155,7 +167,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -164,26 +176,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF4F6EF7"/>
+        <fgColor rgb="FF2F8F5B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F7FF"/>
+        <fgColor rgb="FFF5F2EA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8ECFF"/>
+        <fgColor rgb="FFE6F2EB"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -191,35 +198,23 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -238,8 +233,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Bonnen" displayName="Bonnen" ref="A1:H1" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:H1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="Bonnen" displayName="Bonnen" ref="A1:L1" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:L1">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -248,16 +243,24 @@
     <filterColumn colId="5" hiddenButton="1"/>
     <filterColumn colId="6" hiddenButton="1"/>
     <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+    <filterColumn colId="9" hiddenButton="1"/>
+    <filterColumn colId="10" hiddenButton="1"/>
+    <filterColumn colId="11" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="8">
+  <tableColumns count="12">
     <tableColumn id="1" name="Datum" totalsRowLabel="Total"/>
     <tableColumn id="2" name="Week" totalsRowFunction="none"/>
-    <tableColumn id="3" name="Thema" totalsRowFunction="none"/>
-    <tableColumn id="4" name="Winkel" totalsRowFunction="none"/>
-    <tableColumn id="5" name="Bedrag" totalsRowFunction="none"/>
-    <tableColumn id="6" name="Omschrijving" totalsRowFunction="none"/>
-    <tableColumn id="7" name="Ingescand" totalsRowFunction="none"/>
-    <tableColumn id="8" name="Fingerprint" totalsRowFunction="none"/>
+    <tableColumn id="3" name="Winkel" totalsRowFunction="none"/>
+    <tableColumn id="4" name="Voedsel" totalsRowFunction="none"/>
+    <tableColumn id="5" name="Drank" totalsRowFunction="none"/>
+    <tableColumn id="6" name="Alcohol" totalsRowFunction="none"/>
+    <tableColumn id="7" name="Spelmateriaal" totalsRowFunction="none"/>
+    <tableColumn id="8" name="Knutselgerief" totalsRowFunction="none"/>
+    <tableColumn id="9" name="Kuisproducten" totalsRowFunction="none"/>
+    <tableColumn id="10" name="Varia" totalsRowFunction="none"/>
+    <tableColumn id="11" name="Totaal" totalsRowFunction="none"/>
+    <tableColumn id="12" name="Fingerprint" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -585,43 +588,52 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="12" style="1" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="18" customWidth="1"/>
-    <col min="8" max="8" width="34" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="11" width="14" style="1" customWidth="1"/>
+    <col min="12" max="12" width="34" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -635,212 +647,347 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="1" max="9" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="H2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="I2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="5" t="s">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="B3" s="5">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="C3" s="5">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="D3" s="5">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="E3" s="5">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="F3" s="5">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="G3" s="5">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="H3" s="5">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Opbouw")</f>
+      </c>
+      <c r="I3" s="6">
+        <f>SUM(B3:H3)</f>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 1 (7–11 jul)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C3" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 1 (7–11 jul)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D3" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 1 (7–11 jul)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E3" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 1 (7–11 jul)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F3" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 1 (7–11 jul)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G3" s="8">
-        <f>SUM(B3:F3)</f>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="B4" s="1">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="C4" s="1">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="D4" s="1">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="E4" s="1">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="F4" s="1">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="G4" s="1">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="H4" s="1">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 1")</f>
+      </c>
+      <c r="I4" s="6">
+        <f>SUM(B4:H4)</f>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 2 (14–18 jul)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C4" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 2 (14–18 jul)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D4" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 2 (14–18 jul)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E4" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 2 (14–18 jul)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F4" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 2 (14–18 jul)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G4" s="8">
-        <f>SUM(B4:F4)</f>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="B5" s="5">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="C5" s="5">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="D5" s="5">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="E5" s="5">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="F5" s="5">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="G5" s="5">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="H5" s="5">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 2")</f>
+      </c>
+      <c r="I5" s="6">
+        <f>SUM(B5:H5)</f>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 3 (21–25 jul)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C5" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 3 (21–25 jul)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D5" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 3 (21–25 jul)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E5" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 3 (21–25 jul)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F5" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 3 (21–25 jul)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G5" s="8">
-        <f>SUM(B5:F5)</f>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="1">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="C6" s="1">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="D6" s="1">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="E6" s="1">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="F6" s="1">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="G6" s="1">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="H6" s="1">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 3")</f>
+      </c>
+      <c r="I6" s="6">
+        <f>SUM(B6:H6)</f>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 4 (28 jul–1 aug)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C6" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 4 (28 jul–1 aug)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D6" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 4 (28 jul–1 aug)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E6" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 4 (28 jul–1 aug)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F6" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 4 (28 jul–1 aug)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G6" s="8">
-        <f>SUM(B6:F6)</f>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="5">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="C7" s="5">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="D7" s="5">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="E7" s="5">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="F7" s="5">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="G7" s="5">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="H7" s="5">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 4")</f>
+      </c>
+      <c r="I7" s="6">
+        <f>SUM(B7:H7)</f>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 5 (4–8 aug)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C7" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 5 (4–8 aug)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D7" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 5 (4–8 aug)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E7" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 5 (4–8 aug)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F7" s="7">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 5 (4–8 aug)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G7" s="8">
-        <f>SUM(B7:F7)</f>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="B8" s="1">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="C8" s="1">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="D8" s="1">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="E8" s="1">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="F8" s="1">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="G8" s="1">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="H8" s="1">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 5")</f>
+      </c>
+      <c r="I8" s="6">
+        <f>SUM(B8:H8)</f>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 6 (11–15 aug)",Bonnen[Thema],"Jungle")</f>
-      </c>
-      <c r="C8" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 6 (11–15 aug)",Bonnen[Thema],"Ruimte")</f>
-      </c>
-      <c r="D8" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 6 (11–15 aug)",Bonnen[Thema],"Piraten")</f>
-      </c>
-      <c r="E8" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 6 (11–15 aug)",Bonnen[Thema],"Middeleeuwen")</f>
-      </c>
-      <c r="F8" s="9">
-        <f>SUMIFS(Bonnen[Bedrag],Bonnen[Week],"Week 6 (11–15 aug)",Bonnen[Thema],"Superhelden")</f>
-      </c>
-      <c r="G8" s="8">
-        <f>SUM(B8:F8)</f>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="11">
-        <f>SUM(B3:B8)</f>
-      </c>
-      <c r="C9" s="11">
-        <f>SUM(C3:C8)</f>
-      </c>
-      <c r="D9" s="11">
-        <f>SUM(D3:D8)</f>
-      </c>
-      <c r="E9" s="11">
-        <f>SUM(E3:E8)</f>
-      </c>
-      <c r="F9" s="11">
-        <f>SUM(F3:F8)</f>
-      </c>
-      <c r="G9" s="12">
-        <f>SUM(B9:F9)</f>
+      <c r="B9" s="5">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="C9" s="5">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="D9" s="5">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="E9" s="5">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="F9" s="5">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="G9" s="5">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="H9" s="5">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 6")</f>
+      </c>
+      <c r="I9" s="6">
+        <f>SUM(B9:H9)</f>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" s="1">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="C10" s="1">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="D10" s="1">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="E10" s="1">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="F10" s="1">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="G10" s="1">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="H10" s="1">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Week 7")</f>
+      </c>
+      <c r="I10" s="6">
+        <f>SUM(B10:H10)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" s="5">
+        <f>SUMIFS(Bonnen[Voedsel],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="C11" s="5">
+        <f>SUMIFS(Bonnen[Drank],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="D11" s="5">
+        <f>SUMIFS(Bonnen[Alcohol],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="E11" s="5">
+        <f>SUMIFS(Bonnen[Spelmateriaal],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="F11" s="5">
+        <f>SUMIFS(Bonnen[Knutselgerief],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="G11" s="5">
+        <f>SUMIFS(Bonnen[Kuisproducten],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="H11" s="5">
+        <f>SUMIFS(Bonnen[Varia],Bonnen[Week],"Afbraak")</f>
+      </c>
+      <c r="I11" s="6">
+        <f>SUM(B11:H11)</f>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="8">
+        <f>SUM(B3:B11)</f>
+      </c>
+      <c r="C12" s="8">
+        <f>SUM(C3:C11)</f>
+      </c>
+      <c r="D12" s="8">
+        <f>SUM(D3:D11)</f>
+      </c>
+      <c r="E12" s="8">
+        <f>SUM(E3:E11)</f>
+      </c>
+      <c r="F12" s="8">
+        <f>SUM(F3:F11)</f>
+      </c>
+      <c r="G12" s="8">
+        <f>SUM(G3:G11)</f>
+      </c>
+      <c r="H12" s="8">
+        <f>SUM(H3:H11)</f>
+      </c>
+      <c r="I12" s="9">
+        <f>SUM(B12:H12)</f>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -849,100 +996,115 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="70" customWidth="1"/>
+    <col min="1" max="1" width="78" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>22</v>
+      <c r="A1" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>29</v>
+      <c r="A10" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>31</v>
+      <c r="A13" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>32</v>
+      <c r="A14" s="4" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>9</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
-        <v>33</v>
+      <c r="A16" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>34</v>
+      <c r="A17" s="4" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>